<commit_message>
fix: corrige cortes de nivel v1 para v2 nas formulas da planilha (Versao B); ajustes editoriais guia-validacao e nota-tecnica (auditoria Z)
</commit_message>
<xml_diff>
--- a/public/planilha-validacao-local-mariah.xlsx
+++ b/public/planilha-validacao-local-mariah.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Triagem A↔B" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Painel-resumo" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -2404,7 +2404,7 @@
         <v/>
       </c>
       <c r="K4" s="7" t="str">
-        <f aca="false">IF(J4="","",IF(I4="Sim",  IF(J4&lt;=56,"I",IF(J4&lt;=123,"II",IF(J4&lt;=202,"III","IV"))),  IF(J4&lt;=50,"I",IF(J4&lt;=110,"II",IF(J4&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J4="","",IF(I4="Sim",  IF(J4&lt;=64,"I",IF(J4&lt;=141,"II",IF(J4&lt;=230,"III","IV"))),  IF(J4&lt;=58,"I",IF(J4&lt;=127,"II",IF(J4&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M4" s="6" t="s">
@@ -2435,7 +2435,7 @@
         <v/>
       </c>
       <c r="K5" s="7" t="str">
-        <f aca="false">IF(J5="","",IF(I5="Sim",  IF(J5&lt;=56,"I",IF(J5&lt;=123,"II",IF(J5&lt;=202,"III","IV"))),  IF(J5&lt;=50,"I",IF(J5&lt;=110,"II",IF(J5&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J5="","",IF(I5="Sim",  IF(J5&lt;=64,"I",IF(J5&lt;=141,"II",IF(J5&lt;=230,"III","IV"))),  IF(J5&lt;=58,"I",IF(J5&lt;=127,"II",IF(J5&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M5" s="7" t="s">
@@ -2468,7 +2468,7 @@
         <v/>
       </c>
       <c r="K6" s="7" t="str">
-        <f aca="false">IF(J6="","",IF(I6="Sim",  IF(J6&lt;=56,"I",IF(J6&lt;=123,"II",IF(J6&lt;=202,"III","IV"))),  IF(J6&lt;=50,"I",IF(J6&lt;=110,"II",IF(J6&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J6="","",IF(I6="Sim",  IF(J6&lt;=64,"I",IF(J6&lt;=141,"II",IF(J6&lt;=230,"III","IV"))),  IF(J6&lt;=58,"I",IF(J6&lt;=127,"II",IF(J6&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M6" s="7" t="s">
@@ -2501,7 +2501,7 @@
         <v/>
       </c>
       <c r="K7" s="7" t="str">
-        <f aca="false">IF(J7="","",IF(I7="Sim",  IF(J7&lt;=56,"I",IF(J7&lt;=123,"II",IF(J7&lt;=202,"III","IV"))),  IF(J7&lt;=50,"I",IF(J7&lt;=110,"II",IF(J7&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J7="","",IF(I7="Sim",  IF(J7&lt;=64,"I",IF(J7&lt;=141,"II",IF(J7&lt;=230,"III","IV"))),  IF(J7&lt;=58,"I",IF(J7&lt;=127,"II",IF(J7&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M7" s="7" t="s">
@@ -2534,7 +2534,7 @@
         <v/>
       </c>
       <c r="K8" s="7" t="str">
-        <f aca="false">IF(J8="","",IF(I8="Sim",  IF(J8&lt;=56,"I",IF(J8&lt;=123,"II",IF(J8&lt;=202,"III","IV"))),  IF(J8&lt;=50,"I",IF(J8&lt;=110,"II",IF(J8&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J8="","",IF(I8="Sim",  IF(J8&lt;=64,"I",IF(J8&lt;=141,"II",IF(J8&lt;=230,"III","IV"))),  IF(J8&lt;=58,"I",IF(J8&lt;=127,"II",IF(J8&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M8" s="7" t="s">
@@ -2567,7 +2567,7 @@
         <v/>
       </c>
       <c r="K9" s="7" t="str">
-        <f aca="false">IF(J9="","",IF(I9="Sim",  IF(J9&lt;=56,"I",IF(J9&lt;=123,"II",IF(J9&lt;=202,"III","IV"))),  IF(J9&lt;=50,"I",IF(J9&lt;=110,"II",IF(J9&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J9="","",IF(I9="Sim",  IF(J9&lt;=64,"I",IF(J9&lt;=141,"II",IF(J9&lt;=230,"III","IV"))),  IF(J9&lt;=58,"I",IF(J9&lt;=127,"II",IF(J9&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M9" s="17" t="s">
@@ -2597,7 +2597,7 @@
         <v/>
       </c>
       <c r="K10" s="7" t="str">
-        <f aca="false">IF(J10="","",IF(I10="Sim",  IF(J10&lt;=56,"I",IF(J10&lt;=123,"II",IF(J10&lt;=202,"III","IV"))),  IF(J10&lt;=50,"I",IF(J10&lt;=110,"II",IF(J10&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J10="","",IF(I10="Sim",  IF(J10&lt;=64,"I",IF(J10&lt;=141,"II",IF(J10&lt;=230,"III","IV"))),  IF(J10&lt;=58,"I",IF(J10&lt;=127,"II",IF(J10&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
         <v/>
       </c>
       <c r="K11" s="7" t="str">
-        <f aca="false">IF(J11="","",IF(I11="Sim",  IF(J11&lt;=56,"I",IF(J11&lt;=123,"II",IF(J11&lt;=202,"III","IV"))),  IF(J11&lt;=50,"I",IF(J11&lt;=110,"II",IF(J11&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J11="","",IF(I11="Sim",  IF(J11&lt;=64,"I",IF(J11&lt;=141,"II",IF(J11&lt;=230,"III","IV"))),  IF(J11&lt;=58,"I",IF(J11&lt;=127,"II",IF(J11&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M11" s="10" t="s">
@@ -2646,7 +2646,7 @@
         <v/>
       </c>
       <c r="K12" s="7" t="str">
-        <f aca="false">IF(J12="","",IF(I12="Sim",  IF(J12&lt;=56,"I",IF(J12&lt;=123,"II",IF(J12&lt;=202,"III","IV"))),  IF(J12&lt;=50,"I",IF(J12&lt;=110,"II",IF(J12&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J12="","",IF(I12="Sim",  IF(J12&lt;=64,"I",IF(J12&lt;=141,"II",IF(J12&lt;=230,"III","IV"))),  IF(J12&lt;=58,"I",IF(J12&lt;=127,"II",IF(J12&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M12" s="11" t="s">
@@ -2675,7 +2675,7 @@
         <v/>
       </c>
       <c r="K13" s="7" t="str">
-        <f aca="false">IF(J13="","",IF(I13="Sim",  IF(J13&lt;=56,"I",IF(J13&lt;=123,"II",IF(J13&lt;=202,"III","IV"))),  IF(J13&lt;=50,"I",IF(J13&lt;=110,"II",IF(J13&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J13="","",IF(I13="Sim",  IF(J13&lt;=64,"I",IF(J13&lt;=141,"II",IF(J13&lt;=230,"III","IV"))),  IF(J13&lt;=58,"I",IF(J13&lt;=127,"II",IF(J13&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M13" s="11" t="s">
@@ -2704,7 +2704,7 @@
         <v/>
       </c>
       <c r="K14" s="7" t="str">
-        <f aca="false">IF(J14="","",IF(I14="Sim",  IF(J14&lt;=56,"I",IF(J14&lt;=123,"II",IF(J14&lt;=202,"III","IV"))),  IF(J14&lt;=50,"I",IF(J14&lt;=110,"II",IF(J14&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J14="","",IF(I14="Sim",  IF(J14&lt;=64,"I",IF(J14&lt;=141,"II",IF(J14&lt;=230,"III","IV"))),  IF(J14&lt;=58,"I",IF(J14&lt;=127,"II",IF(J14&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M14" s="11" t="s">
@@ -2733,7 +2733,7 @@
         <v/>
       </c>
       <c r="K15" s="7" t="str">
-        <f aca="false">IF(J15="","",IF(I15="Sim",  IF(J15&lt;=56,"I",IF(J15&lt;=123,"II",IF(J15&lt;=202,"III","IV"))),  IF(J15&lt;=50,"I",IF(J15&lt;=110,"II",IF(J15&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J15="","",IF(I15="Sim",  IF(J15&lt;=64,"I",IF(J15&lt;=141,"II",IF(J15&lt;=230,"III","IV"))),  IF(J15&lt;=58,"I",IF(J15&lt;=127,"II",IF(J15&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M15" s="11" t="s">
@@ -2762,7 +2762,7 @@
         <v/>
       </c>
       <c r="K16" s="7" t="str">
-        <f aca="false">IF(J16="","",IF(I16="Sim",  IF(J16&lt;=56,"I",IF(J16&lt;=123,"II",IF(J16&lt;=202,"III","IV"))),  IF(J16&lt;=50,"I",IF(J16&lt;=110,"II",IF(J16&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J16="","",IF(I16="Sim",  IF(J16&lt;=64,"I",IF(J16&lt;=141,"II",IF(J16&lt;=230,"III","IV"))),  IF(J16&lt;=58,"I",IF(J16&lt;=127,"II",IF(J16&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
       <c r="M16" s="11" t="s">
@@ -2791,7 +2791,7 @@
         <v/>
       </c>
       <c r="K17" s="7" t="str">
-        <f aca="false">IF(J17="","",IF(I17="Sim",  IF(J17&lt;=56,"I",IF(J17&lt;=123,"II",IF(J17&lt;=202,"III","IV"))),  IF(J17&lt;=50,"I",IF(J17&lt;=110,"II",IF(J17&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J17="","",IF(I17="Sim",  IF(J17&lt;=64,"I",IF(J17&lt;=141,"II",IF(J17&lt;=230,"III","IV"))),  IF(J17&lt;=58,"I",IF(J17&lt;=127,"II",IF(J17&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
         <v/>
       </c>
       <c r="K18" s="7" t="str">
-        <f aca="false">IF(J18="","",IF(I18="Sim",  IF(J18&lt;=56,"I",IF(J18&lt;=123,"II",IF(J18&lt;=202,"III","IV"))),  IF(J18&lt;=50,"I",IF(J18&lt;=110,"II",IF(J18&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J18="","",IF(I18="Sim",  IF(J18&lt;=64,"I",IF(J18&lt;=141,"II",IF(J18&lt;=230,"III","IV"))),  IF(J18&lt;=58,"I",IF(J18&lt;=127,"II",IF(J18&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2835,7 +2835,7 @@
         <v/>
       </c>
       <c r="K19" s="7" t="str">
-        <f aca="false">IF(J19="","",IF(I19="Sim",  IF(J19&lt;=56,"I",IF(J19&lt;=123,"II",IF(J19&lt;=202,"III","IV"))),  IF(J19&lt;=50,"I",IF(J19&lt;=110,"II",IF(J19&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J19="","",IF(I19="Sim",  IF(J19&lt;=64,"I",IF(J19&lt;=141,"II",IF(J19&lt;=230,"III","IV"))),  IF(J19&lt;=58,"I",IF(J19&lt;=127,"II",IF(J19&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
         <v/>
       </c>
       <c r="K20" s="7" t="str">
-        <f aca="false">IF(J20="","",IF(I20="Sim",  IF(J20&lt;=56,"I",IF(J20&lt;=123,"II",IF(J20&lt;=202,"III","IV"))),  IF(J20&lt;=50,"I",IF(J20&lt;=110,"II",IF(J20&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J20="","",IF(I20="Sim",  IF(J20&lt;=64,"I",IF(J20&lt;=141,"II",IF(J20&lt;=230,"III","IV"))),  IF(J20&lt;=58,"I",IF(J20&lt;=127,"II",IF(J20&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2879,7 +2879,7 @@
         <v/>
       </c>
       <c r="K21" s="7" t="str">
-        <f aca="false">IF(J21="","",IF(I21="Sim",  IF(J21&lt;=56,"I",IF(J21&lt;=123,"II",IF(J21&lt;=202,"III","IV"))),  IF(J21&lt;=50,"I",IF(J21&lt;=110,"II",IF(J21&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J21="","",IF(I21="Sim",  IF(J21&lt;=64,"I",IF(J21&lt;=141,"II",IF(J21&lt;=230,"III","IV"))),  IF(J21&lt;=58,"I",IF(J21&lt;=127,"II",IF(J21&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="K22" s="7" t="str">
-        <f aca="false">IF(J22="","",IF(I22="Sim",  IF(J22&lt;=56,"I",IF(J22&lt;=123,"II",IF(J22&lt;=202,"III","IV"))),  IF(J22&lt;=50,"I",IF(J22&lt;=110,"II",IF(J22&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J22="","",IF(I22="Sim",  IF(J22&lt;=64,"I",IF(J22&lt;=141,"II",IF(J22&lt;=230,"III","IV"))),  IF(J22&lt;=58,"I",IF(J22&lt;=127,"II",IF(J22&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="K23" s="7" t="str">
-        <f aca="false">IF(J23="","",IF(I23="Sim",  IF(J23&lt;=56,"I",IF(J23&lt;=123,"II",IF(J23&lt;=202,"III","IV"))),  IF(J23&lt;=50,"I",IF(J23&lt;=110,"II",IF(J23&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J23="","",IF(I23="Sim",  IF(J23&lt;=64,"I",IF(J23&lt;=141,"II",IF(J23&lt;=230,"III","IV"))),  IF(J23&lt;=58,"I",IF(J23&lt;=127,"II",IF(J23&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
         <v/>
       </c>
       <c r="K24" s="7" t="str">
-        <f aca="false">IF(J24="","",IF(I24="Sim",  IF(J24&lt;=56,"I",IF(J24&lt;=123,"II",IF(J24&lt;=202,"III","IV"))),  IF(J24&lt;=50,"I",IF(J24&lt;=110,"II",IF(J24&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J24="","",IF(I24="Sim",  IF(J24&lt;=64,"I",IF(J24&lt;=141,"II",IF(J24&lt;=230,"III","IV"))),  IF(J24&lt;=58,"I",IF(J24&lt;=127,"II",IF(J24&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
         <v/>
       </c>
       <c r="K25" s="7" t="str">
-        <f aca="false">IF(J25="","",IF(I25="Sim",  IF(J25&lt;=56,"I",IF(J25&lt;=123,"II",IF(J25&lt;=202,"III","IV"))),  IF(J25&lt;=50,"I",IF(J25&lt;=110,"II",IF(J25&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J25="","",IF(I25="Sim",  IF(J25&lt;=64,"I",IF(J25&lt;=141,"II",IF(J25&lt;=230,"III","IV"))),  IF(J25&lt;=58,"I",IF(J25&lt;=127,"II",IF(J25&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
         <v/>
       </c>
       <c r="K26" s="7" t="str">
-        <f aca="false">IF(J26="","",IF(I26="Sim",  IF(J26&lt;=56,"I",IF(J26&lt;=123,"II",IF(J26&lt;=202,"III","IV"))),  IF(J26&lt;=50,"I",IF(J26&lt;=110,"II",IF(J26&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J26="","",IF(I26="Sim",  IF(J26&lt;=64,"I",IF(J26&lt;=141,"II",IF(J26&lt;=230,"III","IV"))),  IF(J26&lt;=58,"I",IF(J26&lt;=127,"II",IF(J26&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
         <v/>
       </c>
       <c r="K27" s="7" t="str">
-        <f aca="false">IF(J27="","",IF(I27="Sim",  IF(J27&lt;=56,"I",IF(J27&lt;=123,"II",IF(J27&lt;=202,"III","IV"))),  IF(J27&lt;=50,"I",IF(J27&lt;=110,"II",IF(J27&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J27="","",IF(I27="Sim",  IF(J27&lt;=64,"I",IF(J27&lt;=141,"II",IF(J27&lt;=230,"III","IV"))),  IF(J27&lt;=58,"I",IF(J27&lt;=127,"II",IF(J27&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
         <v/>
       </c>
       <c r="K28" s="7" t="str">
-        <f aca="false">IF(J28="","",IF(I28="Sim",  IF(J28&lt;=56,"I",IF(J28&lt;=123,"II",IF(J28&lt;=202,"III","IV"))),  IF(J28&lt;=50,"I",IF(J28&lt;=110,"II",IF(J28&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J28="","",IF(I28="Sim",  IF(J28&lt;=64,"I",IF(J28&lt;=141,"II",IF(J28&lt;=230,"III","IV"))),  IF(J28&lt;=58,"I",IF(J28&lt;=127,"II",IF(J28&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3055,7 +3055,7 @@
         <v/>
       </c>
       <c r="K29" s="7" t="str">
-        <f aca="false">IF(J29="","",IF(I29="Sim",  IF(J29&lt;=56,"I",IF(J29&lt;=123,"II",IF(J29&lt;=202,"III","IV"))),  IF(J29&lt;=50,"I",IF(J29&lt;=110,"II",IF(J29&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J29="","",IF(I29="Sim",  IF(J29&lt;=64,"I",IF(J29&lt;=141,"II",IF(J29&lt;=230,"III","IV"))),  IF(J29&lt;=58,"I",IF(J29&lt;=127,"II",IF(J29&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3077,7 +3077,7 @@
         <v/>
       </c>
       <c r="K30" s="7" t="str">
-        <f aca="false">IF(J30="","",IF(I30="Sim",  IF(J30&lt;=56,"I",IF(J30&lt;=123,"II",IF(J30&lt;=202,"III","IV"))),  IF(J30&lt;=50,"I",IF(J30&lt;=110,"II",IF(J30&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J30="","",IF(I30="Sim",  IF(J30&lt;=64,"I",IF(J30&lt;=141,"II",IF(J30&lt;=230,"III","IV"))),  IF(J30&lt;=58,"I",IF(J30&lt;=127,"II",IF(J30&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3099,7 +3099,7 @@
         <v/>
       </c>
       <c r="K31" s="7" t="str">
-        <f aca="false">IF(J31="","",IF(I31="Sim",  IF(J31&lt;=56,"I",IF(J31&lt;=123,"II",IF(J31&lt;=202,"III","IV"))),  IF(J31&lt;=50,"I",IF(J31&lt;=110,"II",IF(J31&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J31="","",IF(I31="Sim",  IF(J31&lt;=64,"I",IF(J31&lt;=141,"II",IF(J31&lt;=230,"III","IV"))),  IF(J31&lt;=58,"I",IF(J31&lt;=127,"II",IF(J31&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
         <v/>
       </c>
       <c r="K32" s="7" t="str">
-        <f aca="false">IF(J32="","",IF(I32="Sim",  IF(J32&lt;=56,"I",IF(J32&lt;=123,"II",IF(J32&lt;=202,"III","IV"))),  IF(J32&lt;=50,"I",IF(J32&lt;=110,"II",IF(J32&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J32="","",IF(I32="Sim",  IF(J32&lt;=64,"I",IF(J32&lt;=141,"II",IF(J32&lt;=230,"III","IV"))),  IF(J32&lt;=58,"I",IF(J32&lt;=127,"II",IF(J32&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
         <v/>
       </c>
       <c r="K33" s="7" t="str">
-        <f aca="false">IF(J33="","",IF(I33="Sim",  IF(J33&lt;=56,"I",IF(J33&lt;=123,"II",IF(J33&lt;=202,"III","IV"))),  IF(J33&lt;=50,"I",IF(J33&lt;=110,"II",IF(J33&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J33="","",IF(I33="Sim",  IF(J33&lt;=64,"I",IF(J33&lt;=141,"II",IF(J33&lt;=230,"III","IV"))),  IF(J33&lt;=58,"I",IF(J33&lt;=127,"II",IF(J33&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3165,7 +3165,7 @@
         <v/>
       </c>
       <c r="K34" s="7" t="str">
-        <f aca="false">IF(J34="","",IF(I34="Sim",  IF(J34&lt;=56,"I",IF(J34&lt;=123,"II",IF(J34&lt;=202,"III","IV"))),  IF(J34&lt;=50,"I",IF(J34&lt;=110,"II",IF(J34&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J34="","",IF(I34="Sim",  IF(J34&lt;=64,"I",IF(J34&lt;=141,"II",IF(J34&lt;=230,"III","IV"))),  IF(J34&lt;=58,"I",IF(J34&lt;=127,"II",IF(J34&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
         <v/>
       </c>
       <c r="K35" s="7" t="str">
-        <f aca="false">IF(J35="","",IF(I35="Sim",  IF(J35&lt;=56,"I",IF(J35&lt;=123,"II",IF(J35&lt;=202,"III","IV"))),  IF(J35&lt;=50,"I",IF(J35&lt;=110,"II",IF(J35&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J35="","",IF(I35="Sim",  IF(J35&lt;=64,"I",IF(J35&lt;=141,"II",IF(J35&lt;=230,"III","IV"))),  IF(J35&lt;=58,"I",IF(J35&lt;=127,"II",IF(J35&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
         <v/>
       </c>
       <c r="K36" s="7" t="str">
-        <f aca="false">IF(J36="","",IF(I36="Sim",  IF(J36&lt;=56,"I",IF(J36&lt;=123,"II",IF(J36&lt;=202,"III","IV"))),  IF(J36&lt;=50,"I",IF(J36&lt;=110,"II",IF(J36&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J36="","",IF(I36="Sim",  IF(J36&lt;=64,"I",IF(J36&lt;=141,"II",IF(J36&lt;=230,"III","IV"))),  IF(J36&lt;=58,"I",IF(J36&lt;=127,"II",IF(J36&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
         <v/>
       </c>
       <c r="K37" s="7" t="str">
-        <f aca="false">IF(J37="","",IF(I37="Sim",  IF(J37&lt;=56,"I",IF(J37&lt;=123,"II",IF(J37&lt;=202,"III","IV"))),  IF(J37&lt;=50,"I",IF(J37&lt;=110,"II",IF(J37&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J37="","",IF(I37="Sim",  IF(J37&lt;=64,"I",IF(J37&lt;=141,"II",IF(J37&lt;=230,"III","IV"))),  IF(J37&lt;=58,"I",IF(J37&lt;=127,"II",IF(J37&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3253,7 +3253,7 @@
         <v/>
       </c>
       <c r="K38" s="7" t="str">
-        <f aca="false">IF(J38="","",IF(I38="Sim",  IF(J38&lt;=56,"I",IF(J38&lt;=123,"II",IF(J38&lt;=202,"III","IV"))),  IF(J38&lt;=50,"I",IF(J38&lt;=110,"II",IF(J38&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J38="","",IF(I38="Sim",  IF(J38&lt;=64,"I",IF(J38&lt;=141,"II",IF(J38&lt;=230,"III","IV"))),  IF(J38&lt;=58,"I",IF(J38&lt;=127,"II",IF(J38&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
         <v/>
       </c>
       <c r="K39" s="7" t="str">
-        <f aca="false">IF(J39="","",IF(I39="Sim",  IF(J39&lt;=56,"I",IF(J39&lt;=123,"II",IF(J39&lt;=202,"III","IV"))),  IF(J39&lt;=50,"I",IF(J39&lt;=110,"II",IF(J39&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J39="","",IF(I39="Sim",  IF(J39&lt;=64,"I",IF(J39&lt;=141,"II",IF(J39&lt;=230,"III","IV"))),  IF(J39&lt;=58,"I",IF(J39&lt;=127,"II",IF(J39&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
         <v/>
       </c>
       <c r="K40" s="7" t="str">
-        <f aca="false">IF(J40="","",IF(I40="Sim",  IF(J40&lt;=56,"I",IF(J40&lt;=123,"II",IF(J40&lt;=202,"III","IV"))),  IF(J40&lt;=50,"I",IF(J40&lt;=110,"II",IF(J40&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J40="","",IF(I40="Sim",  IF(J40&lt;=64,"I",IF(J40&lt;=141,"II",IF(J40&lt;=230,"III","IV"))),  IF(J40&lt;=58,"I",IF(J40&lt;=127,"II",IF(J40&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
         <v/>
       </c>
       <c r="K41" s="7" t="str">
-        <f aca="false">IF(J41="","",IF(I41="Sim",  IF(J41&lt;=56,"I",IF(J41&lt;=123,"II",IF(J41&lt;=202,"III","IV"))),  IF(J41&lt;=50,"I",IF(J41&lt;=110,"II",IF(J41&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J41="","",IF(I41="Sim",  IF(J41&lt;=64,"I",IF(J41&lt;=141,"II",IF(J41&lt;=230,"III","IV"))),  IF(J41&lt;=58,"I",IF(J41&lt;=127,"II",IF(J41&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
         <v/>
       </c>
       <c r="K42" s="7" t="str">
-        <f aca="false">IF(J42="","",IF(I42="Sim",  IF(J42&lt;=56,"I",IF(J42&lt;=123,"II",IF(J42&lt;=202,"III","IV"))),  IF(J42&lt;=50,"I",IF(J42&lt;=110,"II",IF(J42&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J42="","",IF(I42="Sim",  IF(J42&lt;=64,"I",IF(J42&lt;=141,"II",IF(J42&lt;=230,"III","IV"))),  IF(J42&lt;=58,"I",IF(J42&lt;=127,"II",IF(J42&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3363,7 +3363,7 @@
         <v/>
       </c>
       <c r="K43" s="7" t="str">
-        <f aca="false">IF(J43="","",IF(I43="Sim",  IF(J43&lt;=56,"I",IF(J43&lt;=123,"II",IF(J43&lt;=202,"III","IV"))),  IF(J43&lt;=50,"I",IF(J43&lt;=110,"II",IF(J43&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J43="","",IF(I43="Sim",  IF(J43&lt;=64,"I",IF(J43&lt;=141,"II",IF(J43&lt;=230,"III","IV"))),  IF(J43&lt;=58,"I",IF(J43&lt;=127,"II",IF(J43&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3385,7 +3385,7 @@
         <v/>
       </c>
       <c r="K44" s="7" t="str">
-        <f aca="false">IF(J44="","",IF(I44="Sim",  IF(J44&lt;=56,"I",IF(J44&lt;=123,"II",IF(J44&lt;=202,"III","IV"))),  IF(J44&lt;=50,"I",IF(J44&lt;=110,"II",IF(J44&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J44="","",IF(I44="Sim",  IF(J44&lt;=64,"I",IF(J44&lt;=141,"II",IF(J44&lt;=230,"III","IV"))),  IF(J44&lt;=58,"I",IF(J44&lt;=127,"II",IF(J44&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
         <v/>
       </c>
       <c r="K45" s="7" t="str">
-        <f aca="false">IF(J45="","",IF(I45="Sim",  IF(J45&lt;=56,"I",IF(J45&lt;=123,"II",IF(J45&lt;=202,"III","IV"))),  IF(J45&lt;=50,"I",IF(J45&lt;=110,"II",IF(J45&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J45="","",IF(I45="Sim",  IF(J45&lt;=64,"I",IF(J45&lt;=141,"II",IF(J45&lt;=230,"III","IV"))),  IF(J45&lt;=58,"I",IF(J45&lt;=127,"II",IF(J45&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
         <v/>
       </c>
       <c r="K46" s="7" t="str">
-        <f aca="false">IF(J46="","",IF(I46="Sim",  IF(J46&lt;=56,"I",IF(J46&lt;=123,"II",IF(J46&lt;=202,"III","IV"))),  IF(J46&lt;=50,"I",IF(J46&lt;=110,"II",IF(J46&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J46="","",IF(I46="Sim",  IF(J46&lt;=64,"I",IF(J46&lt;=141,"II",IF(J46&lt;=230,"III","IV"))),  IF(J46&lt;=58,"I",IF(J46&lt;=127,"II",IF(J46&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
         <v/>
       </c>
       <c r="K47" s="7" t="str">
-        <f aca="false">IF(J47="","",IF(I47="Sim",  IF(J47&lt;=56,"I",IF(J47&lt;=123,"II",IF(J47&lt;=202,"III","IV"))),  IF(J47&lt;=50,"I",IF(J47&lt;=110,"II",IF(J47&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J47="","",IF(I47="Sim",  IF(J47&lt;=64,"I",IF(J47&lt;=141,"II",IF(J47&lt;=230,"III","IV"))),  IF(J47&lt;=58,"I",IF(J47&lt;=127,"II",IF(J47&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3473,7 +3473,7 @@
         <v/>
       </c>
       <c r="K48" s="7" t="str">
-        <f aca="false">IF(J48="","",IF(I48="Sim",  IF(J48&lt;=56,"I",IF(J48&lt;=123,"II",IF(J48&lt;=202,"III","IV"))),  IF(J48&lt;=50,"I",IF(J48&lt;=110,"II",IF(J48&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J48="","",IF(I48="Sim",  IF(J48&lt;=64,"I",IF(J48&lt;=141,"II",IF(J48&lt;=230,"III","IV"))),  IF(J48&lt;=58,"I",IF(J48&lt;=127,"II",IF(J48&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
         <v/>
       </c>
       <c r="K49" s="7" t="str">
-        <f aca="false">IF(J49="","",IF(I49="Sim",  IF(J49&lt;=56,"I",IF(J49&lt;=123,"II",IF(J49&lt;=202,"III","IV"))),  IF(J49&lt;=50,"I",IF(J49&lt;=110,"II",IF(J49&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J49="","",IF(I49="Sim",  IF(J49&lt;=64,"I",IF(J49&lt;=141,"II",IF(J49&lt;=230,"III","IV"))),  IF(J49&lt;=58,"I",IF(J49&lt;=127,"II",IF(J49&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
         <v/>
       </c>
       <c r="K50" s="7" t="str">
-        <f aca="false">IF(J50="","",IF(I50="Sim",  IF(J50&lt;=56,"I",IF(J50&lt;=123,"II",IF(J50&lt;=202,"III","IV"))),  IF(J50&lt;=50,"I",IF(J50&lt;=110,"II",IF(J50&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J50="","",IF(I50="Sim",  IF(J50&lt;=64,"I",IF(J50&lt;=141,"II",IF(J50&lt;=230,"III","IV"))),  IF(J50&lt;=58,"I",IF(J50&lt;=127,"II",IF(J50&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3539,7 +3539,7 @@
         <v/>
       </c>
       <c r="K51" s="7" t="str">
-        <f aca="false">IF(J51="","",IF(I51="Sim",  IF(J51&lt;=56,"I",IF(J51&lt;=123,"II",IF(J51&lt;=202,"III","IV"))),  IF(J51&lt;=50,"I",IF(J51&lt;=110,"II",IF(J51&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J51="","",IF(I51="Sim",  IF(J51&lt;=64,"I",IF(J51&lt;=141,"II",IF(J51&lt;=230,"III","IV"))),  IF(J51&lt;=58,"I",IF(J51&lt;=127,"II",IF(J51&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
         <v/>
       </c>
       <c r="K52" s="7" t="str">
-        <f aca="false">IF(J52="","",IF(I52="Sim",  IF(J52&lt;=56,"I",IF(J52&lt;=123,"II",IF(J52&lt;=202,"III","IV"))),  IF(J52&lt;=50,"I",IF(J52&lt;=110,"II",IF(J52&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J52="","",IF(I52="Sim",  IF(J52&lt;=64,"I",IF(J52&lt;=141,"II",IF(J52&lt;=230,"III","IV"))),  IF(J52&lt;=58,"I",IF(J52&lt;=127,"II",IF(J52&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>
@@ -3583,7 +3583,7 @@
         <v/>
       </c>
       <c r="K53" s="7" t="str">
-        <f aca="false">IF(J53="","",IF(I53="Sim",  IF(J53&lt;=56,"I",IF(J53&lt;=123,"II",IF(J53&lt;=202,"III","IV"))),  IF(J53&lt;=50,"I",IF(J53&lt;=110,"II",IF(J53&lt;=180,"III","IV")))))</f>
+        <f aca="false">IF(J53="","",IF(I53="Sim",  IF(J53&lt;=64,"I",IF(J53&lt;=141,"II",IF(J53&lt;=230,"III","IV"))),  IF(J53&lt;=58,"I",IF(J53&lt;=127,"II",IF(J53&lt;=208,"III","IV")))))</f>
         <v/>
       </c>
     </row>

</xml_diff>